<commit_message>
Updating paeper after new identification algorithm was released
</commit_message>
<xml_diff>
--- a/dictionary/variable_dictionary.xlsx
+++ b/dictionary/variable_dictionary.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="420">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="430">
   <si>
     <t xml:space="preserve">File</t>
   </si>
@@ -57,10 +57,10 @@
     <t xml:space="preserve">analysis_sample.parquet</t>
   </si>
   <si>
-    <t xml:space="preserve">8,002,128</t>
-  </si>
-  <si>
-    <t xml:space="preserve">123 MB</t>
+    <t xml:space="preserve">7,764,610</t>
+  </si>
+  <si>
+    <t xml:space="preserve">121 MB</t>
   </si>
   <si>
     <t xml:space="preserve">analysis/code/01_prepare_analysis_data.R</t>
@@ -75,7 +75,7 @@
     <t xml:space="preserve">analysis_origins.parquet</t>
   </si>
   <si>
-    <t xml:space="preserve">179 MB</t>
+    <t xml:space="preserve">180 MB</t>
   </si>
   <si>
     <t xml:space="preserve">Todas as origens, pareadas ou não. Lida por 07 para modelar a seleção na amostra de estimação.</t>
@@ -855,16 +855,46 @@
     <t xml:space="preserve">PNADC (VD4017)</t>
   </si>
   <si>
-    <t xml:space="preserve">Ausente codificado como 0.</t>
+    <t xml:space="preserve">NA quando não informado; ver unpaid_family e income_missing.</t>
   </si>
   <si>
     <t xml:space="preserve">log_income</t>
   </si>
   <si>
-    <t xml:space="preserve">log(1 + income).</t>
+    <t xml:space="preserve">log(1 + income), zero quando income é NA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log(1 + income), zero when income is NA.</t>
   </si>
   <si>
     <t xml:space="preserve">Controle na especificação principal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unpaid_family</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PNADC (VD4009, V4012)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 se trabalhador familiar auxiliar sem remuneração (VD4009 == 10 ou V4012 == 7): renda ausente é um zero verdadeiro.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 if unpaid family worker (VD4009 == 10 or V4012 == 7): missing income is a true zero.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92% dos VD4017 ausentes. Indicador na especificação principal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">income_missing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 se a renda não foi informada e o trabalhador não é familiar auxiliar: não resposta genuína.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 if income is not reported and the worker is not an unpaid family worker: genuine non-response.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicador na especificação principal, separado de unpaid_family.</t>
   </si>
   <si>
     <t xml:space="preserve">1 se o vínculo em t é formal.</t>
@@ -1988,7 +2018,7 @@
         <v>38</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>71</v>
@@ -2008,7 +2038,7 @@
         <v>38</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>74</v>
@@ -2028,7 +2058,7 @@
         <v>77</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>78</v>
@@ -2048,7 +2078,7 @@
         <v>77</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>82</v>
@@ -2887,7 +2917,7 @@
         <v>77</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>223</v>
@@ -3233,87 +3263,87 @@
         <v>281</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>170</v>
+        <v>284</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>77</v>
+        <v>285</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>33</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>33</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>46</v>
+        <v>292</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>290</v>
+        <v>170</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>291</v>
+        <v>77</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>33</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>46</v>
+        <v>295</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>33</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>46</v>
@@ -3321,122 +3351,162 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>263</v>
+        <v>33</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>302</v>
+        <v>46</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>263</v>
+        <v>33</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>302</v>
+        <v>46</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>263</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>77</v>
+        <v>314</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>263</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>33</v>
+        <v>263</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>68</v>
+        <v>319</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>321</v>
+        <v>77</v>
       </c>
       <c r="C35" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D35" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>324</v>
+      <c r="D37" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -3460,21 +3530,21 @@
         <v>22</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>325</v>
+        <v>335</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>326</v>
+        <v>336</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>328</v>
+        <v>338</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>329</v>
+        <v>339</v>
       </c>
     </row>
     <row r="3">
@@ -3482,10 +3552,10 @@
         <v>46</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>330</v>
+        <v>340</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>331</v>
+        <v>341</v>
       </c>
     </row>
     <row r="4">
@@ -3493,10 +3563,10 @@
         <v>46</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
     </row>
     <row r="5">
@@ -3504,10 +3574,10 @@
         <v>46</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>334</v>
+        <v>344</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>335</v>
+        <v>345</v>
       </c>
     </row>
     <row r="6">
@@ -3515,10 +3585,10 @@
         <v>46</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>336</v>
+        <v>346</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>337</v>
+        <v>347</v>
       </c>
     </row>
     <row r="7">
@@ -3526,10 +3596,10 @@
         <v>46</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>338</v>
+        <v>348</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>339</v>
+        <v>349</v>
       </c>
     </row>
     <row r="8">
@@ -3537,10 +3607,10 @@
         <v>46</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>340</v>
+        <v>350</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>341</v>
+        <v>351</v>
       </c>
     </row>
     <row r="9">
@@ -3548,10 +3618,10 @@
         <v>46</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>342</v>
+        <v>352</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>343</v>
+        <v>353</v>
       </c>
     </row>
     <row r="10">
@@ -3559,10 +3629,10 @@
         <v>170</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>344</v>
+        <v>354</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>345</v>
+        <v>355</v>
       </c>
     </row>
     <row r="11">
@@ -3570,10 +3640,10 @@
         <v>174</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>346</v>
+        <v>356</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>347</v>
+        <v>357</v>
       </c>
     </row>
     <row r="12">
@@ -3581,10 +3651,10 @@
         <v>46</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>348</v>
+        <v>358</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>349</v>
+        <v>359</v>
       </c>
     </row>
     <row r="13">
@@ -3592,21 +3662,21 @@
         <v>46</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>350</v>
+        <v>360</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>351</v>
+        <v>361</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>352</v>
+        <v>362</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>353</v>
+        <v>363</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>354</v>
+        <v>364</v>
       </c>
     </row>
     <row r="15">
@@ -3614,10 +3684,10 @@
         <v>46</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>355</v>
+        <v>365</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>356</v>
+        <v>366</v>
       </c>
     </row>
     <row r="16">
@@ -3625,10 +3695,10 @@
         <v>46</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>328</v>
+        <v>338</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>357</v>
+        <v>367</v>
       </c>
     </row>
     <row r="17">
@@ -3636,10 +3706,10 @@
         <v>46</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>330</v>
+        <v>340</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>358</v>
+        <v>368</v>
       </c>
     </row>
     <row r="18">
@@ -3647,10 +3717,10 @@
         <v>46</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>359</v>
+        <v>369</v>
       </c>
     </row>
     <row r="19">
@@ -3658,10 +3728,10 @@
         <v>46</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>340</v>
+        <v>350</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>360</v>
+        <v>370</v>
       </c>
     </row>
     <row r="20">
@@ -3669,10 +3739,10 @@
         <v>137</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>353</v>
+        <v>363</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
     </row>
     <row r="21">
@@ -3680,10 +3750,10 @@
         <v>46</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>355</v>
+        <v>365</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>362</v>
+        <v>372</v>
       </c>
     </row>
     <row r="22">
@@ -3691,10 +3761,10 @@
         <v>46</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>328</v>
+        <v>338</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>363</v>
+        <v>373</v>
       </c>
     </row>
     <row r="23">
@@ -3702,10 +3772,10 @@
         <v>46</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>330</v>
+        <v>340</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>364</v>
+        <v>374</v>
       </c>
     </row>
     <row r="24">
@@ -3713,10 +3783,10 @@
         <v>46</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>365</v>
+        <v>375</v>
       </c>
     </row>
     <row r="25">
@@ -3724,10 +3794,10 @@
         <v>46</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>334</v>
+        <v>344</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>366</v>
+        <v>376</v>
       </c>
     </row>
     <row r="26">
@@ -3735,21 +3805,21 @@
         <v>46</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>336</v>
+        <v>346</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>367</v>
+        <v>377</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>353</v>
+        <v>363</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>369</v>
+        <v>379</v>
       </c>
     </row>
     <row r="28">
@@ -3757,10 +3827,10 @@
         <v>46</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>355</v>
+        <v>365</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>370</v>
+        <v>380</v>
       </c>
     </row>
     <row r="29">
@@ -3768,10 +3838,10 @@
         <v>46</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>328</v>
+        <v>338</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>371</v>
+        <v>381</v>
       </c>
     </row>
     <row r="30">
@@ -3779,21 +3849,21 @@
         <v>46</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>330</v>
+        <v>340</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>372</v>
+        <v>382</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>373</v>
+        <v>383</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>353</v>
+        <v>363</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>374</v>
+        <v>384</v>
       </c>
     </row>
     <row r="32">
@@ -3801,10 +3871,10 @@
         <v>46</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>355</v>
+        <v>365</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>375</v>
+        <v>385</v>
       </c>
     </row>
     <row r="33">
@@ -3812,10 +3882,10 @@
         <v>46</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>328</v>
+        <v>338</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>376</v>
+        <v>386</v>
       </c>
     </row>
     <row r="34">
@@ -3823,10 +3893,10 @@
         <v>46</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>330</v>
+        <v>340</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>377</v>
+        <v>387</v>
       </c>
     </row>
     <row r="35">
@@ -3834,21 +3904,21 @@
         <v>46</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>378</v>
+        <v>388</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>379</v>
+        <v>389</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>381</v>
+        <v>391</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>382</v>
+        <v>392</v>
       </c>
     </row>
     <row r="37">
@@ -3856,10 +3926,10 @@
         <v>46</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>353</v>
+        <v>363</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>383</v>
+        <v>393</v>
       </c>
     </row>
     <row r="38">
@@ -3867,10 +3937,10 @@
         <v>46</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>355</v>
+        <v>365</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>384</v>
+        <v>394</v>
       </c>
     </row>
     <row r="39">
@@ -3878,10 +3948,10 @@
         <v>46</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>328</v>
+        <v>338</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>385</v>
+        <v>395</v>
       </c>
     </row>
     <row r="40">
@@ -3889,10 +3959,10 @@
         <v>46</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>330</v>
+        <v>340</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>386</v>
+        <v>396</v>
       </c>
     </row>
     <row r="41">
@@ -3900,10 +3970,10 @@
         <v>46</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
     </row>
     <row r="42">
@@ -3911,10 +3981,10 @@
         <v>46</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>334</v>
+        <v>344</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>388</v>
+        <v>398</v>
       </c>
     </row>
     <row r="43">
@@ -3922,10 +3992,10 @@
         <v>46</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>336</v>
+        <v>346</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>389</v>
+        <v>399</v>
       </c>
     </row>
     <row r="44">
@@ -3933,10 +4003,10 @@
         <v>46</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>338</v>
+        <v>348</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>390</v>
+        <v>400</v>
       </c>
     </row>
     <row r="45">
@@ -3944,10 +4014,10 @@
         <v>46</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>340</v>
+        <v>350</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>391</v>
+        <v>401</v>
       </c>
     </row>
     <row r="46">
@@ -3955,10 +4025,10 @@
         <v>109</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>392</v>
+        <v>402</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>393</v>
+        <v>403</v>
       </c>
     </row>
     <row r="47">
@@ -3966,10 +4036,10 @@
         <v>112</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>392</v>
+        <v>402</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>394</v>
+        <v>404</v>
       </c>
     </row>
     <row r="48">
@@ -3977,10 +4047,10 @@
         <v>102</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>336</v>
+        <v>346</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>395</v>
+        <v>405</v>
       </c>
     </row>
   </sheetData>
@@ -4000,98 +4070,98 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>396</v>
+        <v>406</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>397</v>
+        <v>407</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>398</v>
+        <v>408</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>399</v>
+        <v>409</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>400</v>
+        <v>410</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>401</v>
+        <v>411</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>402</v>
+        <v>412</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>403</v>
+        <v>413</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>404</v>
+        <v>414</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>405</v>
+        <v>415</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>406</v>
+        <v>416</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>407</v>
+        <v>417</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>408</v>
+        <v>418</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>409</v>
+        <v>419</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>410</v>
+        <v>420</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>411</v>
+        <v>421</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>412</v>
+        <v>422</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>413</v>
+        <v>423</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>414</v>
+        <v>424</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>415</v>
+        <v>425</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>416</v>
+        <v>426</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>417</v>
+        <v>427</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>418</v>
+        <v>428</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
     </row>
   </sheetData>

</xml_diff>